<commit_message>
Automatizacion: Ahora se agregan productos a la BD
</commit_message>
<xml_diff>
--- a/invalidCodes/invalidCodes_Finder.xlsx.xlsx
+++ b/invalidCodes/invalidCodes_Finder.xlsx.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F12"/>
+  <dimension ref="A1:F30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -456,32 +456,32 @@
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>ACTUALIZACIÓN HASTA -- &gt; VIERNES, 19 DE SEPTIEMBRE DE 2025 11:27:15 A. M.</t>
+          <t>ACTUALIZACIÓN HASTA -- &gt; VIERNES, 14 DE NOVIEMBRE DE 2025 03:24:39 P. M.</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>0150230</t>
+          <t>117100121000</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>015.0.230 Supresor de corriente residual. Serie [15, 15Y]</t>
+          <t>DESCONTINUADO, lo reemplaza el producto 11.31.0.024.0000</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>S15</t>
+          <t>S11</t>
         </is>
       </c>
       <c r="D2" t="n">
-        <v>14</v>
+        <v>2</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t xml:space="preserve"> $6,81 </t>
+          <t xml:space="preserve"> $91,19 </t>
         </is>
       </c>
       <c r="F2" t="inlineStr"/>
@@ -489,25 +489,25 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>117100121000</t>
+          <t>1TT182300000</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>DESCONTINUADO, lo reemplaza el producto 11.31.0.024.0000</t>
+          <t>1T.T1.8.230.0000 Termostato p/cajas de pared; 110..230 V AC; Blan</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>S11</t>
+          <t>S1T</t>
         </is>
       </c>
       <c r="D3" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t xml:space="preserve"> $91,19 </t>
+          <t xml:space="preserve"> $64,80 </t>
         </is>
       </c>
       <c r="F3" t="inlineStr"/>
@@ -581,7 +581,7 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>100</v>
+        <v>90</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
@@ -593,12 +593,12 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>623381204040</t>
+          <t>623290244040</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>62.33.8.120.4040 Relé de potencia (120VAC) 3CC 16 A; AgSnO2</t>
+          <t>62.32.9.024.4040 Relé de potencia (24VDC) 2CC 16 A; AgSnO2</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -607,11 +607,11 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>176</v>
+        <v>50</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t xml:space="preserve"> $17,91 </t>
+          <t xml:space="preserve"> $17,06 </t>
         </is>
       </c>
       <c r="F7" t="inlineStr"/>
@@ -619,12 +619,12 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>623382304040</t>
+          <t>623380244040</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>62.33.8.230.4040 Relé de potencia (230VAC) 3CC 16 A; AgSnO2</t>
+          <t>62.33.8.024.4040 Relé de potencia (24VAC) 3CC 16 A; AgSnO2</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -633,11 +633,11 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>130</v>
+        <v>145</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t xml:space="preserve"> $19,03 </t>
+          <t xml:space="preserve"> $17,91 </t>
         </is>
       </c>
       <c r="F8" t="inlineStr"/>
@@ -645,12 +645,12 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>623390124040</t>
+          <t>623381204040</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>62.33.9.012.4040 Relé de potencia (12VDC) 3CC 16 A; AgSnO2</t>
+          <t>62.33.8.120.4040 Relé de potencia (120VAC) 3CC 16 A; AgSnO2</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -659,7 +659,7 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>10</v>
+        <v>396</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
@@ -671,12 +671,12 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>623390244040</t>
+          <t>623382304040</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>62.33.9.024.4040 Relé de potencia (24VDC) 3CC 16 A; AgSnO2</t>
+          <t>62.33.8.230.4040 Relé de potencia (230VAC) 3CC 16 A; AgSnO2</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -685,11 +685,11 @@
         </is>
       </c>
       <c r="D10" t="n">
-        <v>113</v>
+        <v>39</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t xml:space="preserve"> $17,91 </t>
+          <t xml:space="preserve"> $19,03 </t>
         </is>
       </c>
       <c r="F10" t="inlineStr"/>
@@ -697,25 +697,25 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>668282304000</t>
+          <t>623390124040</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>66.82.8.230.4000 Relé de potencia (230VAC) 2CC 30 A; AgSnO2</t>
+          <t>62.33.9.012.4040 Relé de potencia (12VDC) 3CC 16 A; AgSnO2</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>S66</t>
+          <t>S62</t>
         </is>
       </c>
       <c r="D11" t="n">
-        <v>250</v>
+        <v>35</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t xml:space="preserve"> $22,22 </t>
+          <t xml:space="preserve"> $17,91 </t>
         </is>
       </c>
       <c r="F11" t="inlineStr"/>
@@ -723,28 +723,496 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
+          <t>623390244040</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>62.33.9.024.4040 Relé de potencia (24VDC) 3CC 16 A; AgSnO2</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>S62</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>43</v>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> $17,91 </t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>628280244040</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>62.82.8.024.4040 Relé de potencia (24VAC) 2CC 16 A; AgSnO2</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>S62</t>
+        </is>
+      </c>
+      <c r="D13" t="n">
+        <v>5</v>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> $17,32 </t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>668282304000</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>66.82.8.230.4000 Relé de potencia (230VAC) 2CC 30 A; AgSnO2</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>S66</t>
+        </is>
+      </c>
+      <c r="D14" t="n">
+        <v>197</v>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> $22,22 </t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>72B100000500</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>72.B1.0000.1000 Boya Ctrl de nivel líquidos 1CC 10 A; 5m</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>S72</t>
+        </is>
+      </c>
+      <c r="D15" t="n">
+        <v>5</v>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> $84,19 </t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>72B100001000</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>72.B1.0000.1000 Boya Ctrl de nivel líquidos 1CC 10 A; 10m</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>S72</t>
+        </is>
+      </c>
+      <c r="D16" t="n">
+        <v>1</v>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> $105,03 </t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>ATP181100220</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>ATP.1.8.110.0220 1HP, 110V AC, 3Fases, prot. 4-6A, 220V AC</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>SF</t>
+        </is>
+      </c>
+      <c r="D17" t="n">
+        <v>3</v>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> $137,67 </t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>ATP181100440</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>ATP.1.8.110.0440 1HP, 110V AC, 3Fases, prot. 1.6-2.5A, 440V AC</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>SF</t>
+        </is>
+      </c>
+      <c r="D18" t="n">
+        <v>3</v>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> $137,67 </t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>ATP182200440</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>ATP.1.8.220.0440 1HP, 220V AC, 3Fases, prot. 1.6-2.5A, 440V AC</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>SF</t>
+        </is>
+      </c>
+      <c r="D19" t="n">
+        <v>3</v>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> $137,78 </t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>ATP281100220</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>ATP.2.8.110.0220 2HP, 110V AC, 3Fases, prot. 5.5-8A, 220V AC</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>SF</t>
+        </is>
+      </c>
+      <c r="D20" t="n">
+        <v>3</v>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> $140,29 </t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>ATP281100440</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>ATP.2.8.110.0440 2HP, 110V AC, 3Fases, prot. 2.5-4A, 440V AC</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>SF</t>
+        </is>
+      </c>
+      <c r="D21" t="n">
+        <v>3</v>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> $137,67 </t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>ATP282200220</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>ATP.2.8.220.0220 2HP, 220V AC, 3Fases, prot. 5.5-8A, 220V AC</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>SF</t>
+        </is>
+      </c>
+      <c r="D22" t="n">
+        <v>3</v>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> $140,39 </t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>ATP282200440</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>ATP.2.8.220.0440 2HP, 220V AC, 3Fases, prot. 2.5-4A, 440V AC</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>SF</t>
+        </is>
+      </c>
+      <c r="D23" t="n">
+        <v>3</v>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> $137,78 </t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>ATP381100220</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>ATP.3.8.110.0220 3HP, 110V AC, 3Fases, prot. 7-10A, 220V AC</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>SF</t>
+        </is>
+      </c>
+      <c r="D24" t="n">
+        <v>4</v>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> $146,02 </t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>ATP381100440</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>ATP.3.8.110.0440 3HP, 110V AC, 3Fases, prot. 4-6A, 440V AC</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>SF</t>
+        </is>
+      </c>
+      <c r="D25" t="n">
+        <v>4</v>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> $137,67 </t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>ATP382200440</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>ATP.3.8.220.0440 3HP, 220V AC, 3Fases, prot. 4-6A, 440V AC</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>SF</t>
+        </is>
+      </c>
+      <c r="D26" t="n">
+        <v>4</v>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> $137,78 </t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>ATP581100220</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>ATP.5.8.110.0220 5HP, 110V AC, 3Fases, prot. 13-18A, 220V AC</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>SF</t>
+        </is>
+      </c>
+      <c r="D27" t="n">
+        <v>4</v>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> $154,62 </t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr"/>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>ATP581100440</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>ATP.5.8.110.0440 5HP, 110V AC, 3Fases, prot. 5.5-8A, 440V AC</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>SF</t>
+        </is>
+      </c>
+      <c r="D28" t="n">
+        <v>4</v>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> $141,02 </t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>ATP582200440</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>ATP.5.8.220.0440 5HP, 220V AC, 3Fases, prot. 5.5-8A, 440V AC</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>SF</t>
+        </is>
+      </c>
+      <c r="D29" t="n">
+        <v>4</v>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> $141,02 </t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr"/>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
           <t>ZES3046</t>
         </is>
       </c>
-      <c r="B12" t="inlineStr">
+      <c r="B30" t="inlineStr">
         <is>
           <t>Pannel YESLY Demostrative</t>
         </is>
       </c>
-      <c r="C12" t="inlineStr">
+      <c r="C30" t="inlineStr">
         <is>
           <t>S1Y</t>
         </is>
       </c>
-      <c r="D12" t="n">
+      <c r="D30" t="n">
         <v>4</v>
       </c>
-      <c r="E12" t="inlineStr">
+      <c r="E30" t="inlineStr">
         <is>
           <t xml:space="preserve"> $1,02 </t>
         </is>
       </c>
-      <c r="F12" t="inlineStr"/>
+      <c r="F30" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>